<commit_message>
Complete dashboard match history and ADR MVP
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -544,17 +544,17 @@
       <c r="B2" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="n">
-        <v>65</v>
+      <c r="C2" s="3" t="n">
+        <v>100</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>/matches, фильтры, основные колонки, строки из DEM/CSV/JSON</t>
+          <t>/matches, фильтры, сортировка, пагинация, source badges, goal-status filter, match detail page</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Пагинация, сортировка, бейджи источника, полноценная страница деталей матча</t>
+          <t>Только будущая полировка: saved views и export</t>
         </is>
       </c>
       <c r="F2" s="3" t="n">
@@ -567,7 +567,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Улучшать сейчас</t>
+          <t>Готово для текущего MVP</t>
         </is>
       </c>
     </row>
@@ -581,16 +581,16 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>/ с ключевыми метриками, графиком тренда и таблицей карт</t>
+          <t>/ с core stats, trend chart, map stats, data quality, ADR profile, source breakdown, recent session block</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Усилить визуальную иерархию, добавить сводки по сессиям, подписи доверия к данным</t>
+          <t>Только будущая полировка: custom widgets</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
@@ -603,7 +603,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Улучшать сейчас</t>
+          <t>Готово для текущего MVP</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Более надежные маппинги parser events, выбор игрока, фоновые задачи, понятный UX ошибок</t>
+          <t>Parser confidence, player picker, background processing, result screen; см. docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
@@ -675,7 +675,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Топ-приоритет</t>
+          <t>Запланированный топ-приоритет</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Steam/GC/share-code или FACEIT API flow, фоновые jobs</t>
+          <t>Steam/GC/share-code или FACEIT API flow, background jobs; см. docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Позже, но высокая ценность</t>
+          <t>Запланировано</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Accuracy, time-to-damage, crosshair placement, spray metrics</t>
+          <t>Weapon breakdown, timing metrics, confidence, aim dashboard; см. docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Позже, сложно</t>
+          <t>Запланировано</t>
         </is>
       </c>
     </row>
@@ -1265,16 +1265,16 @@
         <v>4</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Работает из DEM player_hurt и CSV/JSON</t>
+          <t>Работает из DEM player_hurt и CSV/JSON; есть dashboard ADR profile, coverage/confidence, recent delta, match-level interpretation</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Валидация урона, исключение team damage, confidence по числу раундов</t>
+          <t>Будущая parser tuning по мере появления новых DEM samples</t>
         </is>
       </c>
       <c r="F22" s="3" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Поддерживать</t>
+          <t>Готово для текущего MVP</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Evidence-backed mistake labels, confidence, examples</t>
+          <t>Structured mistake objects, evidence, confidence, per-match mistakes; см. docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Итеративно сейчас</t>
+          <t>Запланировано</t>
         </is>
       </c>
     </row>
@@ -2529,17 +2529,17 @@
           <t>Match list page</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>65</v>
+      <c r="B9" s="3" t="n">
+        <v>100</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Все игры видны в одном месте</t>
+          <t>Все игры видны в одном месте с sorting, pagination и detail links</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Sorting, pagination, detail page</t>
+          <t>Будущая полировка: saved views/export</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -2554,17 +2554,17 @@
           <t>Match filters</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
-        <v>55</v>
+      <c r="B10" s="3" t="n">
+        <v>100</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Можно фильтровать по map/result/date</t>
+          <t>Фильтры по map/result/source/date/goal status</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Фильтры по source, coach status, imported date</t>
+          <t>Будущая полировка: imported date filter</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -2580,16 +2580,16 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Быстрый обзор формы</t>
+          <t>Core metrics, trends, map stats, data quality, ADR profile, source breakdown</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Больше charts, sessions, explanatory labels</t>
+          <t>Будущая полировка: custom widgets</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2935,7 +2935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3186,6 +3186,30 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>План до 100%</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Обновление</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Dashboard, Match history и ADR доведены до 100% по текущей MVP-шкале; DEM/auto import/aim/mistakes получили пошаговый план.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Codex AI coach handoff provider
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -115,6 +115,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1049,16 +1050,16 @@
         <v>5</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Есть только идея агрегированного payload</t>
+          <t>Provider abstraction, structured coach payload, Codex CLI handoff, prompt bundle</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>OpenAI integration, prompt, safeguards, fallback</t>
+          <t>Сохранение AI-ответа в UI, local_llm provider, structured mistake evidence</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
@@ -2296,6 +2297,42 @@
       <c r="H50" s="2" t="inlineStr">
         <is>
           <t>Позже</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>AI provider abstraction</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>4</v>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>codex_cli_handoff, provider boundary, future local_llm config, docs</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Local LLM execution, result persistence, provider health checks</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>8</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Высокая продуктовая логика: AI coach не зависит от одного model vendor</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Делать сейчас</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2920,6 +2957,31 @@
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Product planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AI coach handoff</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Сайт собирает structured JSON payload и prompt для Codex CLI без OpenAI API key</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Сохранить AI-ответ в UI и подключить local_llm provider</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>AI coach report</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3210,6 +3272,30 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AI architecture</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>docs/AI_COACH_PROVIDER_ARCHITECTURE.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AI update</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Добавлен codex_cli_handoff как текущий мозг и provider boundary для будущей local_llm.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add non-stop development prompts
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -116,6 +116,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -481,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2336,6 +2338,222 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>AI coach result persistence</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>4</v>
+      </c>
+      <c r="C52" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Есть codex_cli_handoff и prompt/payload файлы</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Форма вставки AI-ответа, сохранение в БД, отображение на /coach</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>9</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Ключевой путь к AI-тренеру без OpenAI API</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Делать сейчас</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Multi-category recommendations</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Одна active recommendation и per-match status уже есть</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Категории aim/map/crosshair/grenades/entry/survival, lifecycle, отдельные baselines/targets</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>9</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Главный продуктовый дифференциатор AI coach</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Делать сейчас</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Crosshair placement coach</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>9</v>
+      </c>
+      <c r="C54" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Нет надежных координат/view angles</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Сначала parser evidence: positions/view angles; потом правила и UI</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>8</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Высокий интерес для aim coaching, но data-blocked</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Позже после DEM evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Grenade coach</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>7</v>
+      </c>
+      <c r="C55" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Utility damage, flash assists, enemies flashed best-effort</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Enemy-only flash, duration, lineup/effectiveness, recommendation tracking</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>8</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Высокая coach-ценность для CS2</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>После mistake detection</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Fast post-match refresh</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>8</v>
+      </c>
+      <c r="C56" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Нет автоматического sync</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Import jobs, background scheduler, share-code/demo polling, dedupe</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>9</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Высокая UX-ценность: матч быстро появляется после игры</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>После auth/import scaffold</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Steam OpenID auth</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>5</v>
+      </c>
+      <c r="C57" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Steam OpenID login/linking, user/session model, profile display</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>8</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Нужно для удобного автоимпорта и профиля</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>После DEM stability</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2348,7 +2566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2982,6 +3200,56 @@
       <c r="E25" t="inlineStr">
         <is>
           <t>AI coach report</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Non-stop development prompts</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Есть готовые промты для длинных автономных рабочих сессий</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Поддерживать по мере изменения roadmap</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Developer/product docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Product execution strategy</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Зафиксирован порядок развития AI CS2 Coach</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Обновлять после крупных решений</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Product planning</t>
         </is>
       </c>
     </row>
@@ -2997,7 +3265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3296,6 +3564,78 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Non-stop prompts</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>docs/NON_STOP_DEVELOPMENT_PROMPTS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Product strategy</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>docs/PRODUCT_EXECUTION_STRATEGY.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Steam OpenID source</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://partner.steamgames.com/doc/features/auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Valve match history source</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://developer.valvesoftware.com/wiki/Counter-Strike%3A_Global_Offensive_Access_Match_History</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>FACEIT Data API source</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://docs.faceit.com/docs/data-api/data</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>FACEIT Downloads API source</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://docs.faceit.com/getting-started/Guides/download-api</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Steam auth and import job scaffold
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -1663,17 +1663,17 @@
       <c r="B33" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="C33" s="6" t="n">
-        <v>25</v>
+      <c r="C33" s="4" t="n">
+        <v>45</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Базовое rule-based weakness detection</t>
+          <t>Structured mistake objects, severity, confidence, evidence, coach categories, /coach and match detail UI</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Structured mistake objects, evidence, confidence, per-match mistakes; см. docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
+          <t>Persist mistakes, round-level evidence, feedback loop, AI explanations</t>
         </is>
       </c>
       <c r="F33" s="3" t="n">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Запланировано</t>
+          <t>Итеративно сейчас</t>
         </is>
       </c>
     </row>
@@ -2384,16 +2384,16 @@
         <v>6</v>
       </c>
       <c r="C53" s="8" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Одна active recommendation и per-match status уже есть</t>
+          <t>Coach categories and structured mistakes by aim/map/crosshair/grenades/entry/survival</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Категории aim/map/crosshair/grenades/entry/survival, lifecycle, отдельные baselines/targets</t>
+          <t>Real recommendation lifecycle per category and per-match multi-evaluation</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2456,16 +2456,16 @@
         <v>7</v>
       </c>
       <c r="C55" s="8" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Utility damage, flash assists, enemies flashed best-effort</t>
+          <t>Utility damage/flash fields, grenade mistake cards and match coach section</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Enemy-only flash, duration, lineup/effectiveness, recommendation tracking</t>
+          <t>Enemy-only flash, duration, lineup/effectiveness, confidence</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>После mistake detection</t>
+          <t>После DEM evidence</t>
         </is>
       </c>
     </row>
@@ -2492,16 +2492,16 @@
         <v>8</v>
       </c>
       <c r="C56" s="8" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Нет автоматического sync</t>
+          <t>ImportJob model/statuses and share-code queue scaffold</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Import jobs, background scheduler, share-code/demo polling, dedupe</t>
+          <t>Worker, share-code/demo download, polling, dedupe, status details</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>После auth/import scaffold</t>
+          <t>После Steam hardening</t>
         </is>
       </c>
     </row>
@@ -2527,17 +2527,17 @@
       <c r="B57" t="n">
         <v>5</v>
       </c>
-      <c r="C57" s="8" t="n">
-        <v>0</v>
+      <c r="C57" s="7" t="n">
+        <v>35</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Steam OpenID URL/callback scaffold, SteamAccount model, /settings/imports UI</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Steam OpenID login/linking, user/session model, profile display</t>
+          <t>Production verification, sessions, profile enrichment, security hardening</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>После DEM stability</t>
+          <t>Следующим этапом</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3250,6 +3250,106 @@
       <c r="E27" t="inlineStr">
         <is>
           <t>Product planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Structured mistake detection</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Тренер видит ошибки по категориям с evidence/confidence</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Persist mistakes, round-level evidence, feedback loop</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Mistake detection</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Coach category scorecards</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Aim/map/crosshair/grenades/survival видны как отдельные направления</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Связать с lifecycle рекомендаций</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Multi-category recommendations</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Steam auth scaffold</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Есть Steam OpenID URL/callback scaffold и SteamAccount model</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Hardening OpenID verification, sessions, profile data</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Steam OpenID auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ImportJob scaffold</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Есть очередь import jobs и share-code job creation</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Worker и реальная загрузка demo</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Fast post-match refresh</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3636,6 +3736,18 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Structured mistake detection and Steam auth/import jobs scaffold added. FACEIT kept as future required support.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Persist AI coach reports
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -1051,17 +1051,17 @@
       <c r="B16" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C16" s="6" t="n">
-        <v>20</v>
+      <c r="C16" s="4" t="n">
+        <v>35</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Provider abstraction, structured coach payload, Codex CLI handoff, prompt bundle</t>
+          <t>Provider abstraction, structured payload, Codex handoff, manual AI result persistence</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Сохранение AI-ответа в UI, local_llm provider, structured mistake evidence</t>
+          <t>Automatic local_llm provider and structured AI output</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
@@ -2347,17 +2347,17 @@
       <c r="B52" t="n">
         <v>4</v>
       </c>
-      <c r="C52" s="8" t="n">
-        <v>0</v>
+      <c r="C52" s="7" t="n">
+        <v>55</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Есть codex_cli_handoff и prompt/payload файлы</t>
+          <t>Handoff, paste/save UI, API save endpoint, latest AI report display, report_type/source_ref</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Форма вставки AI-ответа, сохранение в БД, отображение на /coach</t>
+          <t>Автоматический local_llm execution, structured AI sections, feedback loop</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Делать сейчас</t>
+          <t>Продолжать после local_llm provider</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3350,6 +3350,31 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>Fast post-match refresh</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>AI coach result persistence</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>AI report можно сохранить обратно в продукт и открыть на /coach</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Автоматизировать через local_llm provider</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>AI coach report</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add multi-category recommendation tracking
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -2383,17 +2383,17 @@
       <c r="B53" t="n">
         <v>6</v>
       </c>
-      <c r="C53" s="8" t="n">
-        <v>20</v>
+      <c r="C53" s="7" t="n">
+        <v>45</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Coach categories and structured mistakes by aim/map/crosshair/grenades/entry/survival</t>
+          <t>Active goals by survival/aim/grenades/map, per-match evaluations, /coach cards, API, AI payload</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Real recommendation lifecycle per category and per-match multi-evaluation</t>
+          <t>Lifecycle controls, crosshair goal after parser data, tuned thresholds from more demos</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Делать сейчас</t>
+          <t>Продолжать сейчас</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3375,6 +3375,56 @@
       <c r="E32" t="inlineStr">
         <is>
           <t>AI coach report</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Multi-category recommendation tracking</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Есть active goals по survival/aim/grenades/map с green/yellow/red оценкой</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Lifecycle controls и настройка thresholds</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Multi-category recommendations</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Recommendations API</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>GET /api/recommendations отдает все категории прогресса</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Добавить управление status/actions</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Recommendation lifecycle</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3773,6 +3823,18 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Multi-category recommendation tracking added for survival, aim, grenades and map.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add demo import confidence evidence
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -656,16 +656,16 @@
         <v>7</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Реальная загруженная demo попадает в список матчей</t>
+          <t>Real DEM import, duplicate handling, parser confidence, event counts, metric confidence, upload result panel, match detail evidence</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Parser confidence, player picker, background processing, result screen; см. docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
+          <t>Player picker before save, background jobs, deeper side/early timing validation</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
@@ -678,7 +678,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Запланированный топ-приоритет</t>
+          <t>Продолжать сейчас</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Пока fallback на entry deaths</t>
+          <t>Fallback to entry deaths with explicit low confidence warning</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Score by side частично inferred</t>
+          <t>Score by side partially inferred; side stats marked low confidence in parser evidence</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2566,7 +2566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3425,6 +3425,56 @@
       <c r="E34" t="inlineStr">
         <is>
           <t>Recommendation lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DEM parser confidence</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Пользователь видит confidence, event counts, warnings и evidence после DEM import</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Player picker и background processing</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Official DEM upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Match parser evidence panel</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Match detail показывает parser evidence из raw_json</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Round-level parser evidence после deeper parsing</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Match details</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3835,6 +3885,18 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DEM import now stores parser confidence, event counts, metric confidence and warnings.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add local LLM AI provider scaffold
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -1052,16 +1052,16 @@
         <v>5</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Provider abstraction, structured payload, Codex handoff, manual AI result persistence</t>
+          <t>Structured payload, Codex handoff, manual persistence, local_llm direct generation scaffold</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Automatic local_llm provider and structured AI output</t>
+          <t>Real model setup, structured sections, feedback loop, evals</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
@@ -2312,16 +2312,16 @@
         <v>4</v>
       </c>
       <c r="C51" s="7" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>codex_cli_handoff, provider boundary, future local_llm config, docs</t>
+          <t>codex_cli_handoff, local_llm provider scaffold, Ollama/OpenAI-compatible calls, health/generate endpoints</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Local LLM execution, result persistence, provider health checks</t>
+          <t>Real local model setup, streaming, provider UI diagnostics, structured JSON output</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Делать сейчас</t>
+          <t>Продолжать после local model setup</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3475,6 +3475,31 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>Match details</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Local LLM provider scaffold</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Есть Ollama/OpenAI-compatible request path, health и generate endpoints</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Поднять реальную local LLM и добавить streaming/structured JSON</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>AI provider abstraction</t>
         </is>
       </c>
     </row>
@@ -3490,7 +3515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3897,6 +3922,18 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Local LLM provider scaffold added for Ollama and OpenAI-compatible local servers.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add recommendation lifecycle controls
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -2384,16 +2384,16 @@
         <v>6</v>
       </c>
       <c r="C53" s="7" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Active goals by survival/aim/grenades/map, per-match evaluations, /coach cards, API, AI payload</t>
+          <t>Active category goals, per-match evaluations, progress cards, lifecycle controls</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Lifecycle controls, crosshair goal after parser data, tuned thresholds from more demos</t>
+          <t>User-created goals, tuned thresholds, crosshair when parser data exists</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2566,7 +2566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3500,6 +3500,31 @@
       <c r="E37" t="inlineStr">
         <is>
           <t>AI provider abstraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Recommendation lifecycle controls</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Цели можно pause/complete/archive из /coach и API</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>User-created goals, extend/restart/history</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Recommendation lifecycle</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3934,6 +3959,18 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Recommendation lifecycle controls added for pause/complete/archive.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add localized stats and Steam setup
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -118,6 +118,18 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -483,16 +495,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="54" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -588,12 +600,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>/ с core stats, trend chart, map stats, data quality, ADR profile, source breakdown, recent session block</t>
+          <t>/ с core stats, trend chart, map stats, data quality, ADR profile, source breakdown, recent session block; /stats вынесен отдельно</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Только будущая полировка: custom widgets</t>
+          <t>Только будущая полировка: custom widgets и visual polish</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
@@ -728,16 +740,16 @@
         <v>5</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Steam OpenID scaffold, SteamAccount, callback, settings page, Game Authentication Code onboarding; FACEIT пока только в roadmap</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Авторизация, привязка аккаунтов, хранение профиля</t>
+          <t>Hardening OpenID verification, sessions, profile data, FACEIT auth/linking</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
@@ -745,12 +757,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Высокий сигнал: Scope/Leetify используют для онбординга</t>
+          <t>Высокий сигнал: Scope/Leetify используют login для онбординга и автоподгрузки</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Позже, после стабильности DEM</t>
+          <t>Продолжать после Steam worker</t>
         </is>
       </c>
     </row>
@@ -764,16 +776,16 @@
         <v>8</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>ImportJob queue, share-code job, match_history_sync job, Steam auth-code save flow</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Steam/GC/share-code или FACEIT API flow, background jobs; см. docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
+          <t>Реальный worker: Steam match history polling, share code chain, demo download, retries/status UI</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
@@ -786,7 +798,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Запланировано</t>
+          <t>Следующий крупный этап</t>
         </is>
       </c>
     </row>
@@ -2303,254 +2315,326 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>AI provider abstraction</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="C51" s="7" t="n">
+      <c r="C51" s="11" t="n">
         <v>65</v>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="10" t="inlineStr">
         <is>
           <t>codex_cli_handoff, local_llm provider scaffold, Ollama/OpenAI-compatible calls, health/generate endpoints</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E51" s="10" t="inlineStr">
         <is>
           <t>Real local model setup, streaming, provider UI diagnostics, structured JSON output</t>
         </is>
       </c>
-      <c r="F51" t="n">
+      <c r="F51" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G51" s="10" t="inlineStr">
         <is>
           <t>Высокая продуктовая логика: AI coach не зависит от одного model vendor</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H51" s="10" t="inlineStr">
         <is>
           <t>Продолжать после local model setup</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>AI coach result persistence</t>
         </is>
       </c>
-      <c r="B52" t="n">
+      <c r="B52" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="C52" s="7" t="n">
+      <c r="C52" s="11" t="n">
         <v>55</v>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="10" t="inlineStr">
         <is>
           <t>Handoff, paste/save UI, API save endpoint, latest AI report display, report_type/source_ref</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="10" t="inlineStr">
         <is>
           <t>Автоматический local_llm execution, structured AI sections, feedback loop</t>
         </is>
       </c>
-      <c r="F52" t="n">
+      <c r="F52" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G52" s="10" t="inlineStr">
         <is>
           <t>Ключевой путь к AI-тренеру без OpenAI API</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H52" s="10" t="inlineStr">
         <is>
           <t>Продолжать после local_llm provider</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="10" t="inlineStr">
         <is>
           <t>Multi-category recommendations</t>
         </is>
       </c>
-      <c r="B53" t="n">
+      <c r="B53" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="C53" s="7" t="n">
+      <c r="C53" s="11" t="n">
         <v>55</v>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="10" t="inlineStr">
         <is>
           <t>Active category goals, per-match evaluations, progress cards, lifecycle controls</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="10" t="inlineStr">
         <is>
           <t>User-created goals, tuned thresholds, crosshair when parser data exists</t>
         </is>
       </c>
-      <c r="F53" t="n">
+      <c r="F53" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="10" t="inlineStr">
         <is>
           <t>Главный продуктовый дифференциатор AI coach</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H53" s="10" t="inlineStr">
         <is>
           <t>Продолжать сейчас</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t>Crosshair placement coach</t>
         </is>
       </c>
-      <c r="B54" t="n">
+      <c r="B54" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="C54" s="8" t="n">
+      <c r="C54" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="10" t="inlineStr">
         <is>
           <t>Нет надежных координат/view angles</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="10" t="inlineStr">
         <is>
           <t>Сначала parser evidence: positions/view angles; потом правила и UI</t>
         </is>
       </c>
-      <c r="F54" t="n">
+      <c r="F54" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G54" s="10" t="inlineStr">
         <is>
           <t>Высокий интерес для aim coaching, но data-blocked</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H54" s="10" t="inlineStr">
         <is>
           <t>Позже после DEM evidence</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>Grenade coach</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="B55" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="C55" s="8" t="n">
+      <c r="C55" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="10" t="inlineStr">
         <is>
           <t>Utility damage/flash fields, grenade mistake cards and match coach section</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E55" s="10" t="inlineStr">
         <is>
           <t>Enemy-only flash, duration, lineup/effectiveness, confidence</t>
         </is>
       </c>
-      <c r="F55" t="n">
+      <c r="F55" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G55" s="10" t="inlineStr">
         <is>
           <t>Высокая coach-ценность для CS2</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="H55" s="10" t="inlineStr">
         <is>
           <t>После DEM evidence</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>Fast post-match refresh</t>
         </is>
       </c>
-      <c r="B56" t="n">
+      <c r="B56" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="C56" s="8" t="n">
+      <c r="C56" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="10" t="inlineStr">
         <is>
           <t>ImportJob model/statuses and share-code queue scaffold</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E56" s="10" t="inlineStr">
         <is>
           <t>Worker, share-code/demo download, polling, dedupe, status details</t>
         </is>
       </c>
-      <c r="F56" t="n">
+      <c r="F56" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G56" s="10" t="inlineStr">
         <is>
           <t>Высокая UX-ценность: матч быстро появляется после игры</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="H56" s="10" t="inlineStr">
         <is>
           <t>После Steam hardening</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>Steam OpenID auth</t>
         </is>
       </c>
-      <c r="B57" t="n">
+      <c r="B57" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="C57" s="7" t="n">
+      <c r="C57" s="11" t="n">
         <v>35</v>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="10" t="inlineStr">
         <is>
           <t>Steam OpenID URL/callback scaffold, SteamAccount model, /settings/imports UI</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E57" s="10" t="inlineStr">
         <is>
           <t>Production verification, sessions, profile enrichment, security hardening</t>
         </is>
       </c>
-      <c r="F57" t="n">
+      <c r="F57" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="10" t="inlineStr">
         <is>
           <t>Нужно для удобного автоимпорта и профиля</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H57" s="10" t="inlineStr">
         <is>
           <t>Следующим этапом</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>Мультиязычный интерфейс</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>Curated i18n service, RU default, EN switch, translated nav/system labels</t>
+        </is>
+      </c>
+      <c r="E58" s="10" t="inlineStr">
+        <is>
+          <t>Перевести остальные разделы по словарю, добавить fallback QA и language-aware formatting</t>
+        </is>
+      </c>
+      <c r="F58" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G58" s="10" t="inlineStr">
+        <is>
+          <t>Средний сигнал: важно для будущего роста, но RU MVP приоритетнее</t>
+        </is>
+      </c>
+      <c r="H58" s="10" t="inlineStr">
+        <is>
+          <t>Держать как платформенную фичу</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>Отдельная вкладка общей статистики</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" s="10" t="n">
+        <v>75</v>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>/stats с last N/date/all ranges, core metrics, trend, periods, maps, sources, recent matches</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>Metric toggles, export, saved ranges, более красивые charts</t>
+        </is>
+      </c>
+      <c r="F59" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G59" s="10" t="inlineStr">
+        <is>
+          <t>Высокий сигнал: пользователи часто начинают с общей формы и динамики</t>
+        </is>
+      </c>
+      <c r="H59" s="10" t="inlineStr">
+        <is>
+          <t>Доводить вместе с analytics</t>
         </is>
       </c>
     </row>
@@ -2566,14 +2650,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -2610,16 +2694,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Продукт работает как настоящая web panel</t>
+          <t>Продукт работает как настоящая web panel с отдельными разделами и language switch</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Deployment hardening, auth позже</t>
+          <t>Deployment hardening, sessions/auth позже</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -2839,7 +2923,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Core metrics, trends, map stats, data quality, ADR profile, source breakdown</t>
+          <t>Core metrics, trends, map stats, data quality, ADR profile, source breakdown; отдельный /stats появился</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -2860,16 +2944,16 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Показывает прогресс по последним матчам</t>
+          <t>Показывает прогресс по dashboard и /stats</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Metric toggles и time ranges</t>
+          <t>Metric toggles, zoom/time ranges</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -3135,11 +3219,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Проект понятен и воспроизводим</t>
+          <t>Проект понятен и воспроизводим, Steam/i18n/stats описаны</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -3179,352 +3263,427 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>AI coach handoff</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n">
+      <c r="B25" s="11" t="n">
         <v>35</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>Сайт собирает structured JSON payload и prompt для Codex CLI без OpenAI API key</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>Сохранить AI-ответ в UI и подключить local_llm provider</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>AI coach report</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Non-stop development prompts</t>
         </is>
       </c>
-      <c r="B26" s="9" t="n">
+      <c r="B26" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>Есть готовые промты для длинных автономных рабочих сессий</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>Поддерживать по мере изменения roadmap</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>Developer/product docs</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Product execution strategy</t>
         </is>
       </c>
-      <c r="B27" s="9" t="n">
+      <c r="B27" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>Зафиксирован порядок развития AI CS2 Coach</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>Обновлять после крупных решений</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>Product planning</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Structured mistake detection</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n">
+      <c r="B28" s="11" t="n">
         <v>45</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>Тренер видит ошибки по категориям с evidence/confidence</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>Persist mistakes, round-level evidence, feedback loop</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>Mistake detection</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Coach category scorecards</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n">
+      <c r="B29" s="11" t="n">
         <v>35</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>Aim/map/crosshair/grenades/survival видны как отдельные направления</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>Связать с lifecycle рекомендаций</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>Multi-category recommendations</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>Steam auth scaffold</t>
         </is>
       </c>
-      <c r="B30" s="7" t="n">
+      <c r="B30" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Есть Steam OpenID URL/callback, SteamAccount model, settings page и инструкция по Game Authentication Code</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Hardening OpenID verification, sessions, profile data</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Steam OpenID auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>ImportJob scaffold</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Есть Steam OpenID URL/callback scaffold и SteamAccount model</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Hardening OpenID verification, sessions, profile data</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Steam OpenID auth</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>ImportJob scaffold</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="n">
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Есть очередь import jobs, share-code job и match_history_sync job после сохранения auth code</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Worker и реальная загрузка demo</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Fast post-match refresh</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>AI coach result persistence</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>AI report можно сохранить обратно в продукт и открыть на /coach</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Автоматизировать через local_llm provider</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>AI coach report</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Multi-category recommendation tracking</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Есть active goals по survival/aim/grenades/map с green/yellow/red оценкой</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Lifecycle controls и настройка thresholds</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>Multi-category recommendations</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Recommendations API</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>GET /api/recommendations отдает все категории прогресса</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Добавить управление status/actions</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>Recommendation lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>DEM parser confidence</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Пользователь видит confidence, event counts, warnings и evidence после DEM import</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>Player picker и background processing</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>Official DEM upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Match parser evidence panel</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>Match detail показывает parser evidence из raw_json</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Round-level parser evidence после deeper parsing</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>Match details</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Local LLM provider scaffold</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>Есть Ollama/OpenAI-compatible request path, health и generate endpoints</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Поднять реальную local LLM и добавить streaming/structured JSON</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>AI provider abstraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Recommendation lifecycle controls</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>Цели можно pause/complete/archive из /coach и API</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>User-created goals, extend/restart/history</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>Recommendation lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Curated i18n / language switch</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Есть очередь import jobs и share-code job creation</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Worker и реальная загрузка demo</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Fast post-match refresh</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>AI coach result persistence</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="n">
-        <v>55</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>AI report можно сохранить обратно в продукт и открыть на /coach</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Автоматизировать через local_llm provider</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>AI coach report</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Multi-category recommendation tracking</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Есть active goals по survival/aim/grenades/map с green/yellow/red оценкой</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Lifecycle controls и настройка thresholds</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Multi-category recommendations</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Recommendations API</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="n">
-        <v>70</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>GET /api/recommendations отдает все категории прогресса</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Добавить управление status/actions</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Recommendation lifecycle</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>DEM parser confidence</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Пользователь видит confidence, event counts, warnings и evidence после DEM import</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Player picker и background processing</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Official DEM upload</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Match parser evidence panel</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="n">
-        <v>55</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Match detail показывает parser evidence из raw_json</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Round-level parser evidence после deeper parsing</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Match details</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Local LLM provider scaffold</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="n">
-        <v>55</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Есть Ollama/OpenAI-compatible request path, health и generate endpoints</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Поднять реальную local LLM и добавить streaming/structured JSON</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>AI provider abstraction</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Recommendation lifecycle controls</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Цели можно pause/complete/archive из /coach и API</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>User-created goals, extend/restart/history</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Recommendation lifecycle</t>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>Русский интерфейс остается основным, но есть контролируемый путь к EN и другим языкам</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Перевести все шаблоны по словарю, добавить language QA</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>Internationalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Dedicated general stats page</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="n">
+        <v>75</v>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>Можно смотреть форму за последние N матчей, по датам или за всё время</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Metric toggles, saved ranges, export, richer charts</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>General stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Steam Game Authentication Code setup</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>Пользователь понимает, где взять код, может сохранить его и поставить sync job</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Реальный Steam worker, secure secret handling, статус скачивания demos</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Automatic match import</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3702,7 @@
   <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -3792,180 +3951,180 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>План до 100%</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Обновление</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Dashboard, Match history и ADR доведены до 100% по текущей MVP-шкале; DEM/auto import/aim/mistakes получили пошаговый план.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>AI architecture</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>docs/AI_COACH_PROVIDER_ARCHITECTURE.md</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>AI update</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Добавлен codex_cli_handoff как текущий мозг и provider boundary для будущей local_llm.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Non-stop prompts</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>docs/NON_STOP_DEVELOPMENT_PROMPTS.md</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Product strategy</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>docs/PRODUCT_EXECUTION_STRATEGY.md</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Steam OpenID source</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>https://partner.steamgames.com/doc/features/auth</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Valve match history source</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>https://developer.valvesoftware.com/wiki/Counter-Strike%3A_Global_Offensive_Access_Match_History</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>FACEIT Data API source</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>https://docs.faceit.com/docs/data-api/data</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>FACEIT Downloads API source</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>https://docs.faceit.com/getting-started/Guides/download-api</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>Implementation update</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>Structured mistake detection and Steam auth/import jobs scaffold added. FACEIT kept as future required support.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Implementation update</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Multi-category recommendation tracking added for survival, aim, grenades and map.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>Implementation update</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>DEM import now stores parser confidence, event counts, metric confidence and warnings.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Implementation update</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>Local LLM provider scaffold added for Ollama and OpenAI-compatible local servers.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Implementation update</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Recommendation lifecycle controls added for pause/complete/archive.</t>
         </is>

</xml_diff>

<commit_message>
Add Steam match history sync worker
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -740,11 +740,11 @@
         <v>5</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Steam OpenID scaffold, SteamAccount, callback, settings page, Game Authentication Code onboarding; FACEIT пока только в roadmap</t>
+          <t>Steam OpenID scaffold, SteamAccount, callback, settings page, Game Authentication Code onboarding, Steam Web API key storage; FACEIT пока только в roadmap</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -776,16 +776,16 @@
         <v>8</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>ImportJob queue, share-code job, match_history_sync job, Steam auth-code save flow</t>
+          <t>ImportJob queue, share-code job, match_history_sync job, Steam auth-code save flow, GetNextMatchSharingCode worker, steam_history rows</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Реальный worker: Steam match history polling, share code chain, demo download, retries/status UI</t>
+          <t>Demo download по share code, parsing worker, retries/status UI, scheduler</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
@@ -2650,7 +2650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3219,11 +3219,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Проект понятен и воспроизводим, Steam/i18n/stats описаны</t>
+          <t>Проект понятен и воспроизводим, Steam worker/data reset описаны</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -3394,11 +3394,11 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Есть Steam OpenID URL/callback, SteamAccount model, settings page и инструкция по Game Authentication Code</t>
+          <t>Есть Steam OpenID URL/callback, SteamAccount model, settings page, Game Authentication Code и Steam Web API key setup</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
@@ -3419,16 +3419,16 @@
         </is>
       </c>
       <c r="B31" s="12" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Есть очередь import jobs, share-code job и match_history_sync job после сохранения auth code</t>
+          <t>Есть очередь import jobs, share-code job, match_history_sync job и ручной run из UI/API</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Worker и реальная загрузка demo</t>
+          <t>Scheduler, retries, detailed job pages</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -3669,21 +3669,71 @@
         </is>
       </c>
       <c r="B41" s="10" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Пользователь понимает, где взять код, может сохранить его и поставить sync job</t>
+          <t>Пользователь понимает, где взять коды, может сохранить auth code/API key и запустить sync job</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Реальный Steam worker, secure secret handling, статус скачивания demos</t>
+          <t>Реальный demo download по share code, secure secret hardening, статус скачивания demos</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
           <t>Automatic match import</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Steam match-history worker</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>Сервис получает реальные Steam share codes через GetNextMatchSharingCode и сохраняет их как steam_history matches</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Скачать DEM по share code и запустить parser автоматически</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>Automatic match import</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Active data reset for real Steam import</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Тестовые CSV/JSON/ручные DEM матчи удалены из рабочей БД, backup сохранён</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Не требуется; дальше наполнять только настоящими источниками</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>Data hygiene</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prepare public auth and deployment
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2638,6 +2638,78 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>Авторизация пользователя</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C60" s="10" t="n">
+        <v>55</v>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>Landing, регистрация, логин, logout, session cookie, password hashing, protected web UI</t>
+        </is>
+      </c>
+      <c r="E60" s="10" t="inlineStr">
+        <is>
+          <t>Invite/admin flow, password reset, email verification, rate limits, user-owned data isolation</t>
+        </is>
+      </c>
+      <c r="F60" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G60" s="10" t="inlineStr">
+        <is>
+          <t>Высокий сигнал: нужен для публичного продукта и Steam account linking</t>
+        </is>
+      </c>
+      <c r="H60" s="10" t="inlineStr">
+        <is>
+          <t>Продолжать перед публичным запуском</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>Публичный deployment</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C61" s="10" t="n">
+        <v>65</v>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>Nginx reverse proxy, systemd service, domain env, certbot installed, deployment checklist</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>Проброс портов, SSL cert, HTTPS cookies, мониторинг, backups</t>
+        </is>
+      </c>
+      <c r="F61" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G61" s="10" t="inlineStr">
+        <is>
+          <t>Высокий сигнал: без этого нельзя получить Steam API key и дать доступ пользователям</t>
+        </is>
+      </c>
+      <c r="H61" s="10" t="inlineStr">
+        <is>
+          <t>Довести после проброса портов</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2650,7 +2722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3734,6 +3806,106 @@
       <c r="E43" s="10" t="inlineStr">
         <is>
           <t>Data hygiene</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Public landing page</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>Пользователь видит сайт с кнопкой входа до личного кабинета</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Visual polish, pricing/docs/FAQ позже</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>Public website</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Session auth</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="n">
+        <v>55</v>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>Регистрация, вход и закрытые рабочие разделы</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Password reset, email verification, invite/admin, rate limiting</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>User accounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>Nginx reverse proxy</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>Сайт готов принимать внешний HTTP трафик на jcnodex и проксировать FastAPI</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>SSL через certbot после проброса портов</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Systemd service</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>Приложение стартует как сервис и переживает reboot/crash</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>Dedicated user, logs rotation/hardening</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>Deployment</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh roadmap and implementation docs
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Источники и правила" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Матрица фич'!$A$1:$H$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Наши фичи'!$A$1:$E$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Источники и правила'!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Матрица фич'!$A$1:$H$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Наши фичи'!$A$1:$E$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Источники и правила'!$A$1:$B$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -668,7 +668,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -677,7 +677,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Player picker before save, background jobs, deeper side/early timing validation</t>
+          <t>Player picker before save, deeper side/early timing validation, parsed_payload_verified status</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
@@ -740,16 +740,16 @@
         <v>5</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Steam OpenID scaffold, SteamAccount, callback, settings page, Game Authentication Code onboarding, Steam Web API key storage; FACEIT пока только в roadmap</t>
+          <t>Steam OpenID, SteamAccount, callback, settings UI, Game Authentication Code onboarding. FACEIT пока в roadmap.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Hardening OpenID verification, sessions, profile data, FACEIT auth/linking</t>
+          <t>Hardening OpenID verification, profile enrichment, FACEIT auth/linking</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
@@ -762,7 +762,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Продолжать после Steam worker</t>
+          <t>Продолжать после Steam hardening</t>
         </is>
       </c>
     </row>
@@ -776,16 +776,16 @@
         <v>8</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>ImportJob queue, share-code job, match_history_sync job, Steam auth-code save flow, GetNextMatchSharingCode worker, steam_history rows</t>
+          <t>Steam share-code sync, steam_import_all background job, service bot GC resolver, .dem.bz2 download, .dem parse/import, status overview</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Demo download по share code, parsing worker, retries/status UI, scheduler</t>
+          <t>Production scheduler, retries/backoff, FACEIT support, richer job detail page</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
@@ -798,7 +798,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Следующий крупный этап</t>
+          <t>Текущий главный product flow</t>
         </is>
       </c>
     </row>
@@ -2504,16 +2504,16 @@
         <v>8</v>
       </c>
       <c r="C56" s="12" t="n">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>ImportJob model/statuses and share-code queue scaffold</t>
+          <t>steam_import_all queue/background task, immediate page response, overview polling, service bot download/import path</t>
         </is>
       </c>
       <c r="E56" s="10" t="inlineStr">
         <is>
-          <t>Worker, share-code/demo download, polling, dedupe, status details</t>
+          <t>Durable worker process, scheduler, retry/backoff, detailed job page</t>
         </is>
       </c>
       <c r="F56" s="10" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="H56" s="10" t="inlineStr">
         <is>
-          <t>После Steam hardening</t>
+          <t>Продолжать сейчас</t>
         </is>
       </c>
     </row>
@@ -2540,16 +2540,16 @@
         <v>5</v>
       </c>
       <c r="C57" s="11" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>Steam OpenID URL/callback scaffold, SteamAccount model, /settings/imports UI</t>
+          <t>Steam OpenID URL/callback, SteamAccount model, /settings/imports UI, Game Authentication Code onboarding</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
         <is>
-          <t>Production verification, sessions, profile enrichment, security hardening</t>
+          <t>Production callback verification, profile enrichment, security hardening</t>
         </is>
       </c>
       <c r="F57" s="10" t="n">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="H57" s="10" t="inlineStr">
         <is>
-          <t>Следующим этапом</t>
+          <t>Следующим этапом hardening</t>
         </is>
       </c>
     </row>
@@ -2710,8 +2710,44 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Demo storage lifecycle</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>/settings/storage, storage API, manifest, referenced/unreferenced/missing/suspicious classification, future delete candidates</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Approve metric schema, add parsed-payload verification status, then enable raw .dem delete policy</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Высокая операционная ценность после масштабирования auto-import</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Следующим этапом перед raw delete</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H50"/>
+  <autoFilter ref="A1:H62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2722,7 +2758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2891,16 +2927,16 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Реальная CS2 demo превращается в match stats</t>
+          <t>Реальная CS2 demo превращается в match stats; есть confidence, event counts, warnings и evidence</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Parser confidence, background jobs, player picker</t>
+          <t>Player picker before save, deeper side/early timing validation, verified payload status</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -3291,16 +3327,16 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Проект понятен и воспроизводим, Steam worker/data reset описаны</t>
+          <t>Проект понятен и воспроизводим; Steam worker, storage lifecycle и feature roadmap актуализированы</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Обновлять по мере изменений UX</t>
+          <t>Обновлять после каждого крупного UX/architecture изменения</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -3341,16 +3377,16 @@
         </is>
       </c>
       <c r="B25" s="11" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Сайт собирает structured JSON payload и prompt для Codex CLI без OpenAI API key</t>
+          <t>Сайт собирает structured JSON payload и prompt; AI report можно сохранить обратно в продукт; local_llm scaffold есть</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Сохранить AI-ответ в UI и подключить local_llm provider</t>
+          <t>Real local model setup, structured sections, feedback loop</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
@@ -3909,8 +3945,133 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>Steam auth and match-history sync</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>Steam OpenID, Game Authentication Code, latest share code и server-side Steam Web API key позволяют получать Steam share codes</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>Hardening OpenID verification, profile enrichment, FACEIT linking</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="inlineStr">
+        <is>
+          <t>Steam OpenID auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>Steam service bot demo downloader</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="n">
+        <v>75</v>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>Dedicated service bot получает demo URL через CS2 GC, скачивает .dem.bz2, распаковывает и импортирует .dem</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>Stronger bot hardening, retry/backoff, production scheduler</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>Automatic match import</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>ImportJob background worker flow</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>steam_import_all ставится в очередь, web request сразу отвечает, background task делает sync/download/import</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>Durable worker process, retry policy, job detail page</t>
+        </is>
+      </c>
+      <c r="E50" s="10" t="inlineStr">
+        <is>
+          <t>Fast post-match refresh</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>Demo storage lifecycle control</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>/settings/storage, GET /api/storage/demos, manifest, candidates for future raw .dem delete after verified payload</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>Approve metric schema, add verification status, enable delete policy</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>Demo storage lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>Nginx Basic Auth + robots.txt</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>Домен закрыт Basic Auth на время разработки, robots.txt запрещает индексацию</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>HTTPS hardening, monitoring, rate limits</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>Deployment/security</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E24"/>
+  <autoFilter ref="A1:E52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3921,7 +4082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4352,8 +4513,80 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Steam auto-import теперь включает background steam_import_all job, service bot GC resolver, .dem.bz2 download и parse/import.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Demo storage lifecycle добавлен: /settings/storage, API report, manifest, future raw .dem delete candidates; delete policy выключена.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Documentation update</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Roadmap workbook and docs refreshed after inspection on 2026-07-01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Steam architecture</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>docs/STEAM_IMPORT_ARCHITECTURE.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Demo storage TZ</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>docs/DEMO_STORAGE_TZ.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Feature list RU</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>docs/FEATURES_RU.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B21"/>
+  <autoFilter ref="A1:B42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update docs for AI recommendations and aim work
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Источники и правила" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Матрица фич'!$A$1:$H$62</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Наши фичи'!$A$1:$E$52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Источники и правила'!$A$1:$B$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Матрица фич'!$A$1:$H$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Наши фичи'!$A$1:$E$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Источники и правила'!$A$1:$B$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1064,16 +1064,16 @@
         <v>5</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Structured payload, Codex handoff, manual persistence, local_llm direct generation scaffold</t>
+          <t>Provider abstraction, structured payload, Codex handoff, local_llm scaffold, saved AI report with payload snapshot/hash/history</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Real model setup, structured sections, feedback loop, evals</t>
+          <t>Real model setup, structured AI sections, feedback loop/evals</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Следующим этапом</t>
+          <t>Следующим этапом после real model setup</t>
         </is>
       </c>
     </row>
@@ -1136,16 +1136,16 @@
         <v>8</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>HS%, K/D, частично доступны weapon events</t>
+          <t>ADR, K/D, HS%, damage per death, opening duel success, multi-kill rounds, weapon breakdown, data gaps</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Weapon breakdown, timing metrics, confidence, aim dashboard; см. docs/NEXT_100_PERCENT_IMPLEMENTATION_PLAN.md</t>
+          <t>Accuracy/spray/TTK after reliable shot data; dedicated aim dashboard</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
@@ -1153,12 +1153,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Высокий сигнал: Leetify/Refrag и пользователи часто обсуждают aim</t>
+          <t>Leetify/Refrag и пользователи часто обсуждают aim</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Запланировано</t>
+          <t>Продолжать после parser payload</t>
         </is>
       </c>
     </row>
@@ -1172,16 +1172,16 @@
         <v>5</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Entry kills/deaths из первой смерти раунда</t>
+          <t>Entry kills/deaths and opening duel success in aim profile</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Контекст side/map, timing первого контакта, trade context</t>
+          <t>Side/map context, first contact timing, trade context</t>
         </is>
       </c>
       <c r="F19" s="3" t="n">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Высокий сигнал: напрямую actionable</t>
+          <t>Напрямую actionable</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2324,16 +2324,16 @@
         <v>4</v>
       </c>
       <c r="C51" s="11" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>codex_cli_handoff, local_llm provider scaffold, Ollama/OpenAI-compatible calls, health/generate endpoints</t>
+          <t>codex_cli_handoff, local_llm, health/generate endpoints, persistence metadata</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>Real local model setup, streaming, provider UI diagnostics, structured JSON output</t>
+          <t>Streaming, provider UI diagnostics, structured JSON output</t>
         </is>
       </c>
       <c r="F51" s="10" t="n">
@@ -2341,12 +2341,12 @@
       </c>
       <c r="G51" s="10" t="inlineStr">
         <is>
-          <t>Высокая продуктовая логика: AI coach не зависит от одного model vendor</t>
+          <t>AI coach не зависит от одного model vendor</t>
         </is>
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>Продолжать после local model setup</t>
+          <t>Держать как платформенную фичу</t>
         </is>
       </c>
     </row>
@@ -2746,8 +2746,44 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation lifecycle</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Active/paused/completed/archived, extend, restart, category summary, history UI/API</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>User-created goals, restart reason/comments, deeper history charts</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Нужно, когда целей больше одной</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Продолжать после thresholds tuning</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H62"/>
+  <autoFilter ref="A1:H63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2758,7 +2794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3377,11 +3413,11 @@
         </is>
       </c>
       <c r="B25" s="11" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Сайт собирает structured JSON payload и prompt; AI report можно сохранить обратно в продукт; local_llm scaffold есть</t>
+          <t>Structured payload/prompt, saved AI report, payload snapshot/hash/provider metadata/history</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -3552,16 +3588,16 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>AI report можно сохранить обратно в продукт и открыть на /coach</t>
+          <t>AI report хранит markdown, provider metadata, payload hash и payload snapshot; история видна в /coach и API</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>Автоматизировать через local_llm provider</t>
+          <t>Feedback/eval loop, structured AI sections</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
@@ -3577,16 +3613,16 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Есть active goals по survival/aim/grenades/map с green/yellow/red оценкой</t>
+          <t>Survival/aim/grenades/map goals, progress cards, green/yellow/red, extend/restart/history</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>Lifecycle controls и настройка thresholds</t>
+          <t>User-created goals, tuned thresholds, reason comments</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
@@ -3702,16 +3738,16 @@
         </is>
       </c>
       <c r="B38" s="11" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Цели можно pause/complete/archive из /coach и API</t>
+          <t>Pause/complete/archive/extend/restart доступны из /coach и API, есть category summary/history</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>User-created goals, extend/restart/history</t>
+          <t>Goal creation UI, deeper history charts</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
@@ -4070,8 +4106,58 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>Aim profile</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>ADR/KD/HS/opening success/multi-kill/weapon breakdown плюс явные data gaps</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>Accuracy/spray/TTK/crosshair после reliable shot/view/position data</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
+        <is>
+          <t>Aim stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>DEM parser aim payload</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>Parser сохраняет aim_summary, weapon_breakdown и aim_data_gaps в raw_json</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>Round/tick/position timeline, verified payload status</t>
+        </is>
+      </c>
+      <c r="E54" s="10" t="inlineStr">
+        <is>
+          <t>Official DEM upload</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E52"/>
+  <autoFilter ref="A1:E54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4082,7 +4168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4585,8 +4671,68 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>AI coach result persistence now stores payload snapshot/hash/provider metadata and exposes report history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Multi-category recommendations now support extend/restart/history/category summary in UI and API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Aim profile added with honest ADR/KD/HS/opening/multi-kill/weapon breakdown and explicit data gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>Runtime rule</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>After Python route/context or Jinja template changes, restart jc-coach and run authenticated live-smoke pages before final response.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Documentation update</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>AI/recommendations/aim roadmap refreshed on 2026-07-01.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B42"/>
+  <autoFilter ref="A1:B47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update roadmap scoring for deep parser
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -668,16 +668,16 @@
         <v>7</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Real DEM import, duplicate handling, parser confidence, event counts, metric confidence, upload result panel, match detail evidence</t>
+          <t>Real DEM import, duplicate handling, parser confidence, event counts, deep normalized tables, round/player/weapon/damage/duel/grenade storage, match detail deep parser UI</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Player picker before save, deeper side/early timing validation, parsed_payload_verified status</t>
+          <t>Player picker before save, parsed_payload_verified status, side switching validation</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
@@ -1136,16 +1136,16 @@
         <v>8</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ADR, K/D, HS%, damage per death, opening duel success, multi-kill rounds, weapon breakdown, data gaps</t>
+          <t>ADR, K/D, HS%, damage per death, opening duel success, multi-kill rounds, weapon breakdown, estimated accuracy from weapon_fire/player_hurt, deep weapon_stats tables, data gaps</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Accuracy/spray/TTK after reliable shot data; dedicated aim dashboard</t>
+          <t>Spray/TTK/crosshair placement after reliable view-angle/position timeline; dedicated aim drill dashboard</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
@@ -2360,16 +2360,16 @@
         <v>4</v>
       </c>
       <c r="C52" s="11" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Handoff, paste/save UI, API save endpoint, latest AI report display, report_type/source_ref</t>
+          <t>Handoff, paste/save UI, API save endpoint, latest/history AI reports, report_type/source_ref, provider metadata, payload hash/snapshot</t>
         </is>
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>Автоматический local_llm execution, structured AI sections, feedback loop</t>
+          <t>Feedback/eval loop, structured AI sections, automatic local provider execution</t>
         </is>
       </c>
       <c r="F52" s="10" t="n">
@@ -2396,16 +2396,16 @@
         <v>6</v>
       </c>
       <c r="C53" s="11" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>Active category goals, per-match evaluations, progress cards, lifecycle controls</t>
+          <t>Survival/aim/grenades/map goals, per-match evaluations, progress cards, lifecycle controls, history/category summary</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>User-created goals, tuned thresholds, crosshair when parser data exists</t>
+          <t>User-created goals, tuned thresholds, deeper parser-driven thresholds and reason comments</t>
         </is>
       </c>
       <c r="F53" s="10" t="n">
@@ -2720,16 +2720,16 @@
         <v>5</v>
       </c>
       <c r="C62" s="6" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>/settings/storage, storage API, manifest, referenced/unreferenced/missing/suspicious classification, future delete candidates</t>
+          <t>/settings/storage, storage API, manifest, referenced/unreferenced/missing/suspicious classification, future delete candidates, deep parser storage contract documented</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Approve metric schema, add parsed-payload verification status, then enable raw .dem delete policy</t>
+          <t>Add parsed_payload_verified status and explicit retention/delete policy</t>
         </is>
       </c>
       <c r="F62" s="3" t="n">
@@ -2963,16 +2963,16 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Реальная CS2 demo превращается в match stats; есть confidence, event counts, warnings и evidence</t>
+          <t>Реальная CS2 demo превращается в match stats; есть confidence, event counts, warnings, deep parser artifact и normalized evidence</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Player picker before save, deeper side/early timing validation, verified payload status</t>
+          <t>Player picker before save, parsed_payload_verified status, side switching validation</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -3313,16 +3313,16 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Реальная demo участвует в coach-анализе</t>
+          <t>Реальная demo участвует в coach-анализе; есть deep player_rounds, duels, damage и weapon_stats</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>KAST/trade logic, early death timing</t>
+          <t>KAST/trade tuning, side-specific splits</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -3513,16 +3513,16 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Aim/map/crosshair/grenades/survival видны как отдельные направления</t>
+          <t>Aim/map/crosshair/grenades/survival видны как направления и связаны с lifecycle рекомендаций</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Связать с lifecycle рекомендаций</t>
+          <t>User-created goals, thresholds from larger sample</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Survival/aim/grenades/map goals, progress cards, green/yellow/red, extend/restart/history</t>
+          <t>Survival/aim/grenades/map goals, progress cards, green/yellow/red, extend/restart/history/category summary</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -3663,16 +3663,16 @@
         </is>
       </c>
       <c r="B35" s="11" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Пользователь видит confidence, event counts, warnings и evidence после DEM import</t>
+          <t>Пользователь видит confidence, event counts, warnings, evidence и deep parser artifact status</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>Player picker и background processing</t>
+          <t>Player picker и verified payload status</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
@@ -3688,16 +3688,16 @@
         </is>
       </c>
       <c r="B36" s="11" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Match detail показывает parser evidence из raw_json</t>
+          <t>Match detail показывает parser evidence и отдельный блок глубокого DEM parsing: rounds, duels, weapons, grenades</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>Round-level parser evidence после deeper parsing</t>
+          <t>Side-specific round splits and richer timeline UI</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
@@ -4063,16 +4063,16 @@
         </is>
       </c>
       <c r="B51" s="10" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>/settings/storage, GET /api/storage/demos, manifest, candidates for future raw .dem delete after verified payload</t>
+          <t>/settings/storage, API report, manifest, candidates for future raw .dem delete; deep parser contract added; delete policy выключена</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>Approve metric schema, add verification status, enable delete policy</t>
+          <t>Add verification status, enable retention policy</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr">
@@ -4113,16 +4113,16 @@
         </is>
       </c>
       <c r="B53" s="10" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>ADR/KD/HS/opening success/multi-kill/weapon breakdown плюс явные data gaps</t>
+          <t>ADR/KD/HS/opening success/multi-kill/weapon breakdown плюс estimated accuracy и явные data gaps</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>Accuracy/spray/TTK/crosshair после reliable shot/view/position data</t>
+          <t>Spray/TTK/crosshair after reliable shot/view/position data</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
@@ -4138,16 +4138,16 @@
         </is>
       </c>
       <c r="B54" s="10" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Parser сохраняет aim_summary, weapon_breakdown и aim_data_gaps в raw_json</t>
+          <t>Parser сохраняет aim_summary, weapon_breakdown, deep weapon_stats, damage, duels, grenade events and player_rounds</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>Round/tick/position timeline, verified payload status</t>
+          <t>Full tick/view-angle timeline and verified payload status</t>
         </is>
       </c>
       <c r="E54" s="10" t="inlineStr">
@@ -4168,7 +4168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4731,6 +4731,18 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Deep DEM parser added: normalized artifacts/rounds/player_rounds/weapon_stats/damage/duels/grenade_events, match UI, coach overview, production reparse 18 valid artifacts; 52 seven-byte stub files rejected.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Require roadmap update before pushes
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -2756,16 +2756,16 @@
         <v>5</v>
       </c>
       <c r="C63" s="6" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Active/paused/completed/archived, extend, restart, category summary, history UI/API</t>
+          <t>Active/paused/completed/archived, extend, restart, category summary, history UI/API; linked to multi-category recommendation flow</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>User-created goals, restart reason/comments, deeper history charts</t>
+          <t>User-created goals, restart reason/comments, deeper history charts, threshold tuning</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
@@ -4168,7 +4168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4743,6 +4743,18 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Runtime rule</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Перед каждым git push после функциональных изменений Codex должен проверить и при необходимости обновить docs/feature_roadmap_scoring_ru.xlsx и связанный markdown roadmap.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add swing score metric tracking
</commit_message>
<xml_diff>
--- a/docs/feature_roadmap_scoring_ru.xlsx
+++ b/docs/feature_roadmap_scoring_ru.xlsx
@@ -668,11 +668,11 @@
         <v>7</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Real DEM import, duplicate handling, parser confidence, event counts, deep normalized tables, round/player/weapon/damage/duel/grenade storage, match detail deep parser UI</t>
+          <t>Real DEM import, duplicate handling, parser confidence, event counts, swing_score, deep normalized tables, round/player/weapon/damage/duel/grenade storage, match detail deep parser UI</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1136,16 +1136,16 @@
         <v>8</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ADR, K/D, HS%, damage per death, opening duel success, multi-kill rounds, weapon breakdown, estimated accuracy from weapon_fire/player_hurt, deep weapon_stats tables, data gaps</t>
+          <t>ADR, K/D, HS%, damage per death, opening duel success, multi-kill rounds, weapon breakdown, estimated accuracy, swing_score/jc_swing_v1, deep weapon_stats tables, data gaps</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Spray/TTK/crosshair placement after reliable view-angle/position timeline; dedicated aim drill dashboard</t>
+          <t>Spray/TTK/crosshair placement after reliable view-angle/position timeline; dedicated aim/impact dashboard</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
@@ -4113,11 +4113,11 @@
         </is>
       </c>
       <c r="B53" s="10" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>ADR/KD/HS/opening success/multi-kill/weapon breakdown плюс estimated accuracy и явные data gaps</t>
+          <t>ADR/KD/HS/opening success/multi-kill/weapon breakdown плюс estimated accuracy, swing_score и явные data gaps</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
@@ -4138,11 +4138,11 @@
         </is>
       </c>
       <c r="B54" s="10" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Parser сохраняет aim_summary, weapon_breakdown, deep weapon_stats, damage, duels, grenade events and player_rounds</t>
+          <t>Parser сохраняет aim_summary, weapon_breakdown, swing_summary, deep weapon_stats, damage, duels, grenade events and player_rounds</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
@@ -4168,7 +4168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4755,6 +4755,18 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Implementation update</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Swing score added: jc_swing_v1, matches.swing_score, raw_json/artifact swing_summary, UI/API/chart integration, backfill for 18 valid DEM matches.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>